<commit_message>
add testing for Read core logix
</commit_message>
<xml_diff>
--- a/expensesv2/src/main/resources/Repository.xlsx
+++ b/expensesv2/src/main/resources/Repository.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Formação\workspaceV2\expensesV2\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346A5D1E-97D4-4182-80A5-EEAE52EE0B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383A6210-1CB3-4431-9535-4776F1BA74D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{14EC8011-9132-421C-BEF6-A483E0F6AAD9}"/>
+    <workbookView xWindow="2970" yWindow="1920" windowWidth="14400" windowHeight="7270" activeTab="2" xr2:uid="{14EC8011-9132-421C-BEF6-A483E0F6AAD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -71,9 +71,6 @@
     <t>typeid</t>
   </si>
   <si>
-    <t xml:space="preserve">isRevenue </t>
-  </si>
-  <si>
     <t>user_id</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>1.4</t>
+  </si>
+  <si>
+    <t>isRevenue</t>
   </si>
 </sst>
 </file>
@@ -480,7 +480,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -491,10 +491,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -545,7 +545,7 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -559,7 +559,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -576,7 +576,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -594,7 +594,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
         <v>5</v>
@@ -606,6 +606,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B2DFD334E6A3034F898C07A5B179AF82" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4b47bed1f976da8d6b40dd0f87550b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xmlns:ns4="e24bc939-ed6e-4865-8a4d-2519bddf4458" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="58236cf1faf4b8c1ff480fa16364175a" ns3:_="" ns4:_="">
     <xsd:import namespace="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
@@ -852,24 +869,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6C94329-D6A5-498C-999E-67C6D3CED00A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -886,29 +911,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>